<commit_message>
update upload feature and voucher detail
</commit_message>
<xml_diff>
--- a/wwwroot/assets/doc_form/product_upload_format.xlsx
+++ b/wwwroot/assets/doc_form/product_upload_format.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="26130"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\iHishab\iHishab\wwwroot\assets\doc_form\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFAF75B9-A6E8-4FD7-AD43-C31852CB39B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A4468FE-4B7A-41A7-8A2F-546B5AF966F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,14 +20,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>Product Name</t>
   </si>
   <si>
-    <t>Descriptive Name</t>
-  </si>
-  <si>
     <t>Quantity Unit</t>
   </si>
   <si>
@@ -38,6 +35,18 @@
   </si>
   <si>
     <t>Avg Price</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Other Name</t>
+  </si>
+  <si>
+    <t>Brand No</t>
+  </si>
+  <si>
+    <t>Part No</t>
   </si>
 </sst>
 </file>
@@ -59,7 +68,7 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -394,40 +403,52 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F1"/>
-  <sheetFormatPr defaultColWidth="51" defaultRowHeight="14.4"/>
+  <dimension ref="A1:I1"/>
+  <sheetFormatPr defaultColWidth="51" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="2" width="51" customWidth="1"/>
-    <col min="3" max="3" width="16.6640625" customWidth="1"/>
-    <col min="4" max="4" width="20.33203125" style="4" customWidth="1"/>
-    <col min="5" max="5" width="18.6640625" style="4" customWidth="1"/>
-    <col min="6" max="6" width="17.109375" style="4" customWidth="1"/>
-    <col min="7" max="7" width="51" customWidth="1"/>
+    <col min="1" max="1" width="51" customWidth="1"/>
+    <col min="2" max="2" width="26.42578125" customWidth="1"/>
+    <col min="3" max="3" width="34.5703125" customWidth="1"/>
+    <col min="4" max="4" width="36.85546875" customWidth="1"/>
+    <col min="5" max="5" width="16.7109375" customWidth="1"/>
+    <col min="6" max="6" width="20.28515625" style="4" customWidth="1"/>
+    <col min="7" max="7" width="18.7109375" style="4" customWidth="1"/>
+    <col min="8" max="8" width="17.140625" style="4" customWidth="1"/>
+    <col min="9" max="9" width="51" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="1" customFormat="1" ht="22.2" customHeight="1">
+    <row r="1" spans="1:9" s="1" customFormat="1" ht="22.15" customHeight="1">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="F1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="I1" s="2" t="s">
         <v>5</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"PC(S),KG(S),SET,PACKET,LITTER,METER,DOZEN,FEET,INCH,CM"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
update product upload file
</commit_message>
<xml_diff>
--- a/wwwroot/assets/doc_form/product_upload_format.xlsx
+++ b/wwwroot/assets/doc_form/product_upload_format.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\iHishab\iHishab\wwwroot\assets\doc_form\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F39CE1BC-9138-46AC-9B65-F4C6748D9AAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6323EC23-EDE8-445B-9636-960F98621E5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -43,9 +43,6 @@
     <t>Other Name</t>
   </si>
   <si>
-    <t>Brand No</t>
-  </si>
-  <si>
     <t>Part No</t>
   </si>
   <si>
@@ -53,6 +50,9 @@
   </si>
   <si>
     <t>Country of Origin</t>
+  </si>
+  <si>
+    <t>Brand</t>
   </si>
 </sst>
 </file>
@@ -431,10 +431,10 @@
         <v>6</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>1</v>
@@ -452,10 +452,10 @@
         <v>5</v>
       </c>
       <c r="J1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="K1" s="2" t="s">
         <v>9</v>
-      </c>
-      <c r="K1" s="2" t="s">
-        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>